<commit_message>
Provider Happy Path Fix 9.2.0
</commit_message>
<xml_diff>
--- a/config/testdata/testdata.xlsx
+++ b/config/testdata/testdata.xlsx
@@ -1,23 +1,24 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30527"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MMHNZ_V2_AUTOMATION\config\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BE28E80-82CA-49D3-BA05-317F7BD9ABD3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{413A7987-2A7C-4190-ACAB-5FEB54A02C42}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="2" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Happy_Path_Patient_Web_and_MR" sheetId="1" r:id="rId1"/>
-    <sheet name="Sanity_Patient_Web" sheetId="5" r:id="rId2"/>
-    <sheet name="Happy_Path_Patient_Mobile_App" sheetId="2" r:id="rId3"/>
-    <sheet name="General_Sanity_Provider_Web" sheetId="3" r:id="rId4"/>
-    <sheet name="Happy_Path_Provider_Web" sheetId="4" r:id="rId5"/>
+    <sheet name="Alex_Happy_Path_Web_and_MR" sheetId="6" r:id="rId2"/>
+    <sheet name="Sanity_Patient_Web" sheetId="5" r:id="rId3"/>
+    <sheet name="Happy_Path_Patient_Mobile_App" sheetId="2" r:id="rId4"/>
+    <sheet name="General_Sanity_Provider_Web" sheetId="3" r:id="rId5"/>
+    <sheet name="Happy_Path_Provider_Web" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2967" uniqueCount="1526">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3022" uniqueCount="1561">
   <si>
     <t>KEY</t>
   </si>
@@ -4620,13 +4621,118 @@
   </si>
   <si>
     <t>https://v2portalhotfix.mmh-demo.com/home</t>
+  </si>
+  <si>
+    <t>PRD</t>
+  </si>
+  <si>
+    <t>Alex Appointments</t>
+  </si>
+  <si>
+    <t>Rainbow Medical Centre;Myself;A new issue;My usual provider;Evo_3_46_Dev_Loc1;Dr B Beta;AFTER_THREE_DAYS;In-person;WheelChair</t>
+  </si>
+  <si>
+    <t>Alex prod;Myself;A new issue;My usual provider;Alex Prod Loc2;GP2;AFTER_THREE_DAYS;In-person;WheelChair</t>
+  </si>
+  <si>
+    <t>ALEX_VISIT_APPOINTMENT_DETAILS</t>
+  </si>
+  <si>
+    <t>In-person;Appointment is for Yourself;A new issue;15 minutes;48 Market Place Auckland Central Auckland 1050</t>
+  </si>
+  <si>
+    <t>In-person;Appointment is for Yourself;A new issue;15 minutes;175 FernBrook Close East Tamaki Manukau 2013</t>
+  </si>
+  <si>
+    <t>ALEX_VISIT_APPOINTMENT_SUMMARY</t>
+  </si>
+  <si>
+    <t>Approved;Dr B Beta;AFTER_THREE_DAYS;A new issue|Wheel Chair</t>
+  </si>
+  <si>
+    <t>Approved;GP2;AFTER_THREE_DAYS;A new issue|Wheel Chair</t>
+  </si>
+  <si>
+    <t>Evo_3_46_Dev_HC;Myself;A new issue;By provider;Dr B Beta;Evo_3_46_Dev_Loc1;AFTER_THREE_DAYS;Video;WheelChair</t>
+  </si>
+  <si>
+    <t>Alex prod;Myself;A new issue;By doctor;GP2;Alex Prod Loc2;AFTER_THREE_DAYS;Video;WheelChair</t>
+  </si>
+  <si>
+    <t>ALEX_VIDEO_APPOINTMENT_DETAILS</t>
+  </si>
+  <si>
+    <t>Video;Appointment is for Yourself;A new issue;15 minutes;48 Market Place Auckland Central Auckland 1050</t>
+  </si>
+  <si>
+    <t>Video;Appointment is for Yourself;A new issue;15 minutes;175 FernBrook Close East Tamaki Manukau 2013</t>
+  </si>
+  <si>
+    <t>ALEX_VIDEO_APPOINTMENT_SUMMARY</t>
+  </si>
+  <si>
+    <t>BOOK_FLEXIBLE_SLOT_PHONE_APPOINTMENT</t>
+  </si>
+  <si>
+    <t>Evo_3_46_Dev_HC;Myself;A new issue;By earliest available;Evo_3_46_Dev_Loc1;Evo_3_46_Dev_Loc1;TODAY;Dr B Beta;Phone;WheelChair;210913528</t>
+  </si>
+  <si>
+    <t>Alex prod;Myself;A new issue;By earliest available;Alex Prod Loc2;Alex Prod Loc2;TODAY;GP2;Phone;WheelChair;210913528</t>
+  </si>
+  <si>
+    <t>ALEX_PHONE_APPOINTMENT_DETAILS</t>
+  </si>
+  <si>
+    <t>Phone;Appointment is for Yourself;A new issue;15 minutes;48 Market Place Auckland Central Auckland 1050</t>
+  </si>
+  <si>
+    <t>Phone;Appointment is for Yourself;A new issue;15 minutes;175 FernBrook Close East Tamaki Manukau 2013</t>
+  </si>
+  <si>
+    <t>ALEX_PHONE_APPOINTMENT_SUMMARY</t>
+  </si>
+  <si>
+    <t>Approved;Dr B Beta;TODAY;A new issue|Wheel Chair</t>
+  </si>
+  <si>
+    <t>Approved;GP2;TODAY;A new issue|Wheel Chair</t>
+  </si>
+  <si>
+    <t>TODAY_DATE</t>
+  </si>
+  <si>
+    <t>TODAY</t>
+  </si>
+  <si>
+    <t>BOOK_FLEXIBLE_SLOT_VISIT_APPOINTMENT_BY_LOCATION</t>
+  </si>
+  <si>
+    <t>Evo_3_46_Dev_HC;Myself;A new issue;By location;Evo_3_46_Dev_Loc1;Dr B Beta;AFTER_THREE_DAYS;In-person;WheelChair;Evo_3_46_Dev_Loc1</t>
+  </si>
+  <si>
+    <t>Alex prod;Myself;A new issue;By location;Alex Prod Loc2;GP2;AFTER_THREE_DAYS;In-person;WheelChair;Alex Prod Loc2</t>
+  </si>
+  <si>
+    <t>Approved;GP2;AFTER_THREE_DAYS</t>
+  </si>
+  <si>
+    <t>Cancelled;GP2;AFTER_THREE_DAYS</t>
+  </si>
+  <si>
+    <t>Select Script Urgency;Urgent/Same day - Std Fee: $1,022.00 (Incl. GST);Next Day - Std Fee: $1,033.00 (Incl. GST);48 Hours - Std Fee: $1,044.00 (Incl. GST);72 Hours - Std Fee: $1,055.00 (Incl. GST)</t>
+  </si>
+  <si>
+    <t>Automation1_Loc1;Gp2White;Send Script to Pharmacy;Select from my saved list;Addington Pharmacy;Auckland Central;Addington Pharmacy;48 Hours;Trasylol 500,000KIU/50ml Inj;Repeat Medication Testing for Sent Script by Pharmacy;Addington Pharmacy</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> 536 Mount Albert Road, Three Kings, Auckland&lt;br/&gt; Phone: (09) 625 3838 </t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="29">
+  <fonts count="30">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -4808,6 +4914,13 @@
       <name val="Segoe UI"/>
       <family val="2"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Verdana"/>
+      <family val="2"/>
+    </font>
   </fonts>
   <fills count="13">
     <fill>
@@ -4883,7 +4996,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="18">
+  <borders count="19">
     <border>
       <left/>
       <right/>
@@ -5124,6 +5237,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
@@ -5131,7 +5259,7 @@
     <xf numFmtId="0" fontId="24" fillId="0" borderId="9"/>
     <xf numFmtId="0" fontId="26" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="107">
+  <cellXfs count="119">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -5403,6 +5531,28 @@
     </xf>
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="29" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="18" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="9" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="4" fillId="0" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="8" fillId="11" borderId="18" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="4">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
@@ -17695,6 +17845,632 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7FA9EBCD-2DF9-4062-BB11-B0836A43559F}">
+  <dimension ref="A1:W20"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="37.5703125" customWidth="1"/>
+    <col min="2" max="2" width="42.42578125" customWidth="1"/>
+    <col min="3" max="3" width="52.28515625" customWidth="1"/>
+    <col min="4" max="4" width="56" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A1" s="107" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="108" t="s">
+        <v>1077</v>
+      </c>
+      <c r="C1" s="109" t="s">
+        <v>1</v>
+      </c>
+      <c r="D1" s="108" t="s">
+        <v>1526</v>
+      </c>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+      <c r="G1" s="2"/>
+      <c r="H1" s="2"/>
+      <c r="I1" s="2"/>
+      <c r="J1" s="2"/>
+      <c r="K1" s="2"/>
+      <c r="L1" s="2"/>
+      <c r="M1" s="2"/>
+      <c r="N1" s="2"/>
+      <c r="O1" s="2"/>
+      <c r="P1" s="2"/>
+      <c r="Q1" s="2"/>
+      <c r="R1" s="2"/>
+      <c r="S1" s="2"/>
+      <c r="T1" s="2"/>
+      <c r="U1" s="2"/>
+      <c r="V1" s="2"/>
+      <c r="W1" s="2"/>
+    </row>
+    <row r="2" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A2" s="110"/>
+      <c r="B2" s="111" t="s">
+        <v>1527</v>
+      </c>
+      <c r="C2" s="110"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+      <c r="H2" s="2"/>
+      <c r="I2" s="2"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="2"/>
+      <c r="L2" s="2"/>
+      <c r="M2" s="2"/>
+      <c r="N2" s="2"/>
+      <c r="O2" s="2"/>
+      <c r="P2" s="2"/>
+      <c r="Q2" s="2"/>
+      <c r="R2" s="2"/>
+      <c r="S2" s="2"/>
+      <c r="T2" s="2"/>
+      <c r="U2" s="2"/>
+      <c r="V2" s="2"/>
+      <c r="W2" s="2"/>
+    </row>
+    <row r="3" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A3" s="112"/>
+      <c r="B3" s="112"/>
+      <c r="C3" s="113"/>
+      <c r="D3" s="108"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2"/>
+      <c r="K3" s="2"/>
+      <c r="L3" s="2"/>
+      <c r="M3" s="2"/>
+      <c r="N3" s="2"/>
+      <c r="O3" s="2"/>
+      <c r="P3" s="2"/>
+      <c r="Q3" s="2"/>
+      <c r="R3" s="2"/>
+      <c r="S3" s="2"/>
+      <c r="T3" s="2"/>
+      <c r="U3" s="2"/>
+      <c r="V3" s="2"/>
+      <c r="W3" s="2"/>
+    </row>
+    <row r="4" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A4" s="114" t="s">
+        <v>923</v>
+      </c>
+      <c r="B4" s="114" t="s">
+        <v>1528</v>
+      </c>
+      <c r="C4" s="114" t="s">
+        <v>1529</v>
+      </c>
+      <c r="D4" s="115" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+      <c r="H4" s="2"/>
+      <c r="I4" s="2"/>
+      <c r="J4" s="2"/>
+      <c r="K4" s="2"/>
+      <c r="L4" s="2"/>
+      <c r="M4" s="2"/>
+      <c r="N4" s="2"/>
+      <c r="O4" s="2"/>
+      <c r="P4" s="2"/>
+      <c r="Q4" s="2"/>
+      <c r="R4" s="2"/>
+      <c r="S4" s="2"/>
+      <c r="T4" s="2"/>
+      <c r="U4" s="2"/>
+      <c r="V4" s="2"/>
+      <c r="W4" s="2"/>
+    </row>
+    <row r="5" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A5" s="107" t="s">
+        <v>1530</v>
+      </c>
+      <c r="B5" s="107" t="s">
+        <v>1531</v>
+      </c>
+      <c r="C5" s="107" t="s">
+        <v>1532</v>
+      </c>
+      <c r="D5" s="107" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+      <c r="H5" s="2"/>
+      <c r="I5" s="2"/>
+      <c r="J5" s="2"/>
+      <c r="K5" s="2"/>
+      <c r="L5" s="2"/>
+      <c r="M5" s="2"/>
+      <c r="N5" s="2"/>
+      <c r="O5" s="2"/>
+      <c r="P5" s="2"/>
+      <c r="Q5" s="2"/>
+      <c r="R5" s="2"/>
+      <c r="S5" s="2"/>
+      <c r="T5" s="2"/>
+      <c r="U5" s="2"/>
+      <c r="V5" s="2"/>
+      <c r="W5" s="2"/>
+    </row>
+    <row r="6" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A6" s="107" t="s">
+        <v>1533</v>
+      </c>
+      <c r="B6" s="107" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C6" s="107" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D6" s="107" t="s">
+        <v>914</v>
+      </c>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
+      <c r="I6" s="2"/>
+      <c r="J6" s="2"/>
+      <c r="K6" s="2"/>
+      <c r="L6" s="2"/>
+      <c r="M6" s="2"/>
+      <c r="N6" s="2"/>
+      <c r="O6" s="2"/>
+      <c r="P6" s="2"/>
+      <c r="Q6" s="2"/>
+      <c r="R6" s="2"/>
+      <c r="S6" s="2"/>
+      <c r="T6" s="2"/>
+      <c r="U6" s="2"/>
+      <c r="V6" s="2"/>
+      <c r="W6" s="2"/>
+    </row>
+    <row r="7" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A7" s="116"/>
+      <c r="B7" s="116"/>
+      <c r="C7" s="116"/>
+      <c r="D7" s="108"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2"/>
+      <c r="K7" s="2"/>
+      <c r="L7" s="2"/>
+      <c r="M7" s="2"/>
+      <c r="N7" s="2"/>
+      <c r="O7" s="2"/>
+      <c r="P7" s="2"/>
+      <c r="Q7" s="2"/>
+      <c r="R7" s="2"/>
+      <c r="S7" s="2"/>
+      <c r="T7" s="2"/>
+      <c r="U7" s="2"/>
+      <c r="V7" s="2"/>
+      <c r="W7" s="2"/>
+    </row>
+    <row r="8" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A8" s="115" t="s">
+        <v>924</v>
+      </c>
+      <c r="B8" s="115" t="s">
+        <v>1536</v>
+      </c>
+      <c r="C8" s="115" t="s">
+        <v>1537</v>
+      </c>
+      <c r="D8" s="115" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+      <c r="H8" s="2"/>
+      <c r="I8" s="2"/>
+      <c r="J8" s="2"/>
+      <c r="K8" s="2"/>
+      <c r="L8" s="2"/>
+      <c r="M8" s="2"/>
+      <c r="N8" s="2"/>
+      <c r="O8" s="2"/>
+      <c r="P8" s="2"/>
+      <c r="Q8" s="2"/>
+      <c r="R8" s="2"/>
+      <c r="S8" s="2"/>
+      <c r="T8" s="2"/>
+      <c r="U8" s="2"/>
+      <c r="V8" s="2"/>
+      <c r="W8" s="2"/>
+    </row>
+    <row r="9" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A9" s="116" t="s">
+        <v>1538</v>
+      </c>
+      <c r="B9" s="116" t="s">
+        <v>1539</v>
+      </c>
+      <c r="C9" s="116" t="s">
+        <v>1540</v>
+      </c>
+      <c r="D9" s="108"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+      <c r="H9" s="2"/>
+      <c r="I9" s="2"/>
+      <c r="J9" s="2"/>
+      <c r="K9" s="2"/>
+      <c r="L9" s="2"/>
+      <c r="M9" s="2"/>
+      <c r="N9" s="2"/>
+      <c r="O9" s="2"/>
+      <c r="P9" s="2"/>
+      <c r="Q9" s="2"/>
+      <c r="R9" s="2"/>
+      <c r="S9" s="2"/>
+      <c r="T9" s="2"/>
+      <c r="U9" s="2"/>
+      <c r="V9" s="2"/>
+      <c r="W9" s="2"/>
+    </row>
+    <row r="10" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A10" s="107" t="s">
+        <v>1541</v>
+      </c>
+      <c r="B10" s="107" t="s">
+        <v>1534</v>
+      </c>
+      <c r="C10" s="107" t="s">
+        <v>1535</v>
+      </c>
+      <c r="D10" s="107" t="s">
+        <v>25</v>
+      </c>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+      <c r="H10" s="2"/>
+      <c r="I10" s="2"/>
+      <c r="J10" s="2"/>
+      <c r="K10" s="2"/>
+      <c r="L10" s="2"/>
+      <c r="M10" s="2"/>
+      <c r="N10" s="2"/>
+      <c r="O10" s="2"/>
+      <c r="P10" s="2"/>
+      <c r="Q10" s="2"/>
+      <c r="R10" s="2"/>
+      <c r="S10" s="2"/>
+      <c r="T10" s="2"/>
+      <c r="U10" s="2"/>
+      <c r="V10" s="2"/>
+      <c r="W10" s="2"/>
+    </row>
+    <row r="11" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A11" s="117"/>
+      <c r="B11" s="117"/>
+      <c r="C11" s="117"/>
+      <c r="D11" s="108"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+      <c r="H11" s="2"/>
+      <c r="I11" s="2"/>
+      <c r="J11" s="2"/>
+      <c r="K11" s="2"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="2"/>
+      <c r="N11" s="2"/>
+      <c r="O11" s="2"/>
+      <c r="P11" s="2"/>
+      <c r="Q11" s="2"/>
+      <c r="R11" s="2"/>
+      <c r="S11" s="2"/>
+      <c r="T11" s="2"/>
+      <c r="U11" s="2"/>
+      <c r="V11" s="2"/>
+      <c r="W11" s="2"/>
+    </row>
+    <row r="12" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A12" s="115" t="s">
+        <v>1542</v>
+      </c>
+      <c r="B12" s="115" t="s">
+        <v>1543</v>
+      </c>
+      <c r="C12" s="115" t="s">
+        <v>1544</v>
+      </c>
+      <c r="D12" s="115" t="s">
+        <v>1002</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+      <c r="H12" s="2"/>
+      <c r="I12" s="2"/>
+      <c r="J12" s="2"/>
+      <c r="K12" s="2"/>
+      <c r="L12" s="2"/>
+      <c r="M12" s="2"/>
+      <c r="N12" s="2"/>
+      <c r="O12" s="2"/>
+      <c r="P12" s="2"/>
+      <c r="Q12" s="2"/>
+      <c r="R12" s="2"/>
+      <c r="S12" s="2"/>
+      <c r="T12" s="2"/>
+      <c r="U12" s="2"/>
+      <c r="V12" s="2"/>
+      <c r="W12" s="2"/>
+    </row>
+    <row r="13" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A13" s="116" t="s">
+        <v>1545</v>
+      </c>
+      <c r="B13" s="116" t="s">
+        <v>1546</v>
+      </c>
+      <c r="C13" s="116" t="s">
+        <v>1547</v>
+      </c>
+      <c r="D13" s="108"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+      <c r="H13" s="2"/>
+      <c r="I13" s="2"/>
+      <c r="J13" s="2"/>
+      <c r="K13" s="2"/>
+      <c r="L13" s="2"/>
+      <c r="M13" s="2"/>
+      <c r="N13" s="2"/>
+      <c r="O13" s="2"/>
+      <c r="P13" s="2"/>
+      <c r="Q13" s="2"/>
+      <c r="R13" s="2"/>
+      <c r="S13" s="2"/>
+      <c r="T13" s="2"/>
+      <c r="U13" s="2"/>
+      <c r="V13" s="2"/>
+      <c r="W13" s="2"/>
+    </row>
+    <row r="14" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A14" s="107" t="s">
+        <v>1548</v>
+      </c>
+      <c r="B14" s="107" t="s">
+        <v>1549</v>
+      </c>
+      <c r="C14" s="107" t="s">
+        <v>1550</v>
+      </c>
+      <c r="D14" s="107" t="s">
+        <v>25</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+      <c r="H14" s="2"/>
+      <c r="I14" s="2"/>
+      <c r="J14" s="2"/>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2"/>
+      <c r="M14" s="2"/>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2"/>
+      <c r="Q14" s="2"/>
+      <c r="R14" s="2"/>
+      <c r="S14" s="2"/>
+      <c r="T14" s="2"/>
+      <c r="U14" s="2"/>
+      <c r="V14" s="2"/>
+      <c r="W14" s="2"/>
+    </row>
+    <row r="15" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A15" s="107" t="s">
+        <v>1551</v>
+      </c>
+      <c r="B15" s="107" t="s">
+        <v>1552</v>
+      </c>
+      <c r="C15" s="107" t="s">
+        <v>1552</v>
+      </c>
+      <c r="D15" s="107" t="s">
+        <v>1552</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+      <c r="H15" s="2"/>
+      <c r="I15" s="2"/>
+      <c r="J15" s="2"/>
+      <c r="K15" s="2"/>
+      <c r="L15" s="2"/>
+      <c r="M15" s="2"/>
+      <c r="N15" s="2"/>
+      <c r="O15" s="2"/>
+      <c r="P15" s="2"/>
+      <c r="Q15" s="2"/>
+      <c r="R15" s="2"/>
+      <c r="S15" s="2"/>
+      <c r="T15" s="2"/>
+      <c r="U15" s="2"/>
+      <c r="V15" s="2"/>
+      <c r="W15" s="2"/>
+    </row>
+    <row r="16" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A16" s="116"/>
+      <c r="B16" s="116"/>
+      <c r="C16" s="118"/>
+      <c r="D16" s="108"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+      <c r="H16" s="2"/>
+      <c r="I16" s="2"/>
+      <c r="J16" s="2"/>
+      <c r="K16" s="2"/>
+      <c r="L16" s="2"/>
+      <c r="M16" s="2"/>
+      <c r="N16" s="2"/>
+      <c r="O16" s="2"/>
+      <c r="P16" s="2"/>
+      <c r="Q16" s="2"/>
+      <c r="R16" s="2"/>
+      <c r="S16" s="2"/>
+      <c r="T16" s="2"/>
+      <c r="U16" s="2"/>
+      <c r="V16" s="2"/>
+      <c r="W16" s="2"/>
+    </row>
+    <row r="17" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A17" s="116"/>
+      <c r="B17" s="116"/>
+      <c r="C17" s="118"/>
+      <c r="D17" s="108"/>
+      <c r="E17" s="2"/>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+      <c r="H17" s="2"/>
+      <c r="I17" s="2"/>
+      <c r="J17" s="2"/>
+      <c r="K17" s="2"/>
+      <c r="L17" s="2"/>
+      <c r="M17" s="2"/>
+      <c r="N17" s="2"/>
+      <c r="O17" s="2"/>
+      <c r="P17" s="2"/>
+      <c r="Q17" s="2"/>
+      <c r="R17" s="2"/>
+      <c r="S17" s="2"/>
+      <c r="T17" s="2"/>
+      <c r="U17" s="2"/>
+      <c r="V17" s="2"/>
+      <c r="W17" s="2"/>
+    </row>
+    <row r="18" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A18" s="114" t="s">
+        <v>1553</v>
+      </c>
+      <c r="B18" s="114" t="s">
+        <v>1554</v>
+      </c>
+      <c r="C18" s="114" t="s">
+        <v>1555</v>
+      </c>
+      <c r="D18" s="115" t="s">
+        <v>1009</v>
+      </c>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+      <c r="H18" s="2"/>
+      <c r="I18" s="2"/>
+      <c r="J18" s="2"/>
+      <c r="K18" s="2"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="2"/>
+      <c r="N18" s="2"/>
+      <c r="O18" s="2"/>
+      <c r="P18" s="2"/>
+      <c r="Q18" s="2"/>
+      <c r="R18" s="2"/>
+      <c r="S18" s="2"/>
+      <c r="T18" s="2"/>
+      <c r="U18" s="2"/>
+      <c r="V18" s="2"/>
+      <c r="W18" s="2"/>
+    </row>
+    <row r="19" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A19" s="107" t="s">
+        <v>44</v>
+      </c>
+      <c r="B19" s="107" t="s">
+        <v>46</v>
+      </c>
+      <c r="C19" s="109" t="s">
+        <v>1556</v>
+      </c>
+      <c r="D19" s="107" t="s">
+        <v>45</v>
+      </c>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+      <c r="H19" s="2"/>
+      <c r="I19" s="2"/>
+      <c r="J19" s="2"/>
+      <c r="K19" s="2"/>
+      <c r="L19" s="2"/>
+      <c r="M19" s="2"/>
+      <c r="N19" s="2"/>
+      <c r="O19" s="2"/>
+      <c r="P19" s="2"/>
+      <c r="Q19" s="2"/>
+      <c r="R19" s="2"/>
+      <c r="S19" s="2"/>
+      <c r="T19" s="2"/>
+      <c r="U19" s="2"/>
+      <c r="V19" s="2"/>
+      <c r="W19" s="2"/>
+    </row>
+    <row r="20" spans="1:23" ht="13.5" customHeight="1">
+      <c r="A20" s="107" t="s">
+        <v>47</v>
+      </c>
+      <c r="B20" s="107" t="s">
+        <v>49</v>
+      </c>
+      <c r="C20" s="109" t="s">
+        <v>1557</v>
+      </c>
+      <c r="D20" s="107" t="s">
+        <v>48</v>
+      </c>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+      <c r="H20" s="2"/>
+      <c r="I20" s="2"/>
+      <c r="J20" s="2"/>
+      <c r="K20" s="2"/>
+      <c r="L20" s="2"/>
+      <c r="M20" s="2"/>
+      <c r="N20" s="2"/>
+      <c r="O20" s="2"/>
+      <c r="P20" s="2"/>
+      <c r="Q20" s="2"/>
+      <c r="R20" s="2"/>
+      <c r="S20" s="2"/>
+      <c r="T20" s="2"/>
+      <c r="U20" s="2"/>
+      <c r="V20" s="2"/>
+      <c r="W20" s="2"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -17744,7 +18520,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="56" t="s">
-        <v>1050</v>
+        <v>1525</v>
       </c>
       <c r="C2" s="50" t="s">
         <v>980</v>
@@ -22452,7 +23228,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:V1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
@@ -32374,7 +33150,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:Z1000"/>
   <sheetFormatPr defaultColWidth="14.42578125" defaultRowHeight="15" customHeight="1"/>
@@ -34232,7 +35008,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -34266,7 +35042,7 @@
         <v>2</v>
       </c>
       <c r="B2" s="96" t="s">
-        <v>1050</v>
+        <v>1525</v>
       </c>
       <c r="C2" s="71" t="s">
         <v>980</v>
@@ -34478,13 +35254,13 @@
         <v>412</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>413</v>
-      </c>
-      <c r="C18" s="61" t="s">
-        <v>413</v>
+        <v>1558</v>
+      </c>
+      <c r="C18" s="9" t="s">
+        <v>1558</v>
       </c>
       <c r="D18" s="9" t="s">
-        <v>413</v>
+        <v>1558</v>
       </c>
     </row>
     <row r="19" spans="1:4" ht="15.75" thickBot="1">
@@ -34562,7 +35338,7 @@
         <v>425</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>426</v>
+        <v>1560</v>
       </c>
       <c r="C24" s="61" t="s">
         <v>1241</v>
@@ -34888,7 +35664,7 @@
         <v>72</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>453</v>
+        <v>1559</v>
       </c>
       <c r="C56" s="59" t="s">
         <v>73</v>

</xml_diff>